<commit_message>
docs(cliente): planilha devolutiva com as 3 listas e o motivo de cada OS
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QsRs6rpRETaPHmRZKdtg1Y
</commit_message>
<xml_diff>
--- a/docs/cliente/2026-10-15-divergencias-os-devolutiva.xlsx
+++ b/docs/cliente/2026-10-15-divergencias-os-devolutiva.xlsx
@@ -4,15 +4,16 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="OS no HUB e não no Field" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Outras listas" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="No HUB e não no Field" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="No Field e não no HUB" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="Nem no HUB nem no Field" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="148">
   <si>
     <t>OS</t>
   </si>
@@ -26,10 +27,10 @@
     <t>Nº da OS no Field</t>
   </si>
   <si>
-    <t>Situação</t>
-  </si>
-  <si>
-    <t>Consideração</t>
+    <t>Motivo</t>
+  </si>
+  <si>
+    <t>Explicação</t>
   </si>
   <si>
     <t>O que fazer</t>
@@ -44,13 +45,13 @@
     <t>HUB</t>
   </si>
   <si>
-    <t>Existe nos dois sistemas</t>
-  </si>
-  <si>
-    <t>No Field, a atividade desta OS está ARQUIVADA. Por isso ela não aparece no relatório do Field. No hub está em "pendente faturamento".</t>
-  </si>
-  <si>
-    <t>Confirmar com a equipe se o arquivamento foi de propósito. Se o serviço não acabou, desarquivar a atividade no Field.</t>
+    <t>Atividade arquivada no Field</t>
+  </si>
+  <si>
+    <t>Existe no hub (pendente faturamento) e no Field, mas a atividade dela está arquivada no Field. Por isso não aparece no relatório de lá.</t>
+  </si>
+  <si>
+    <t>Confirmar se o arquivamento foi de propósito. Se o serviço não acabou, desarquivar no Field.</t>
   </si>
   <si>
     <t>1026-006374</t>
@@ -59,7 +60,10 @@
     <t>341</t>
   </si>
   <si>
-    <t>No Field, esta OS está com o número 341. O número 1026-006374 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
+    <t>Número diferente nos dois</t>
+  </si>
+  <si>
+    <t>No Field esta OS está com o número 341. O número 1026-006374 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
   </si>
   <si>
     <t>Procurar no Field pela OS 341 (ou pelo campo "OS Cliente"). Nada a corrigir.</t>
@@ -71,7 +75,7 @@
     <t>822</t>
   </si>
   <si>
-    <t>No Field, esta OS está com o número 822. O número 0726-018976 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
+    <t>No Field esta OS está com o número 822. O número 0726-018976 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
   </si>
   <si>
     <t>Procurar no Field pela OS 822 (ou pelo campo "OS Cliente"). Nada a corrigir.</t>
@@ -83,7 +87,7 @@
     <t>766</t>
   </si>
   <si>
-    <t>No Field, esta OS está com o número 766. O número 1026-007524 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
+    <t>No Field esta OS está com o número 766. O número 1026-007524 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
   </si>
   <si>
     <t>Procurar no Field pela OS 766 (ou pelo campo "OS Cliente"). Nada a corrigir.</t>
@@ -95,7 +99,7 @@
     <t>266</t>
   </si>
   <si>
-    <t>No Field, esta OS está com o número 266. O número 0926-014930 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
+    <t>No Field esta OS está com o número 266. O número 0926-014930 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
   </si>
   <si>
     <t>Procurar no Field pela OS 266 (ou pelo campo "OS Cliente"). Nada a corrigir.</t>
@@ -107,7 +111,7 @@
     <t>54</t>
   </si>
   <si>
-    <t>No Field, esta OS está com o número 54. O número 0526-014042 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
+    <t>No Field esta OS está com o número 54. O número 0526-014042 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
   </si>
   <si>
     <t>Procurar no Field pela OS 54 (ou pelo campo "OS Cliente"). Nada a corrigir.</t>
@@ -119,23 +123,347 @@
     <t>347</t>
   </si>
   <si>
-    <t>No Field, esta OS está com o número 347. O número 0726-019256 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
+    <t>No Field esta OS está com o número 347. O número 0726-019256 está no campo "OS Cliente" dela, e é esse que o hub mostra. Por isso o PROCV não encontrou.</t>
   </si>
   <si>
     <t>Procurar no Field pela OS 347 (ou pelo campo "OS Cliente"). Nada a corrigir.</t>
   </si>
   <si>
-    <t>As listas "OS nem no HUB e nem no Field" e "OS no Field e não no HUB" não chegaram até nós (os prints enviados eram iguais ao da primeira lista).</t>
-  </si>
-  <si>
-    <t>Se puderem mandar, conferimos e devolvemos no mesmo formato.</t>
+    <t>Coluna1</t>
+  </si>
+  <si>
+    <t>Coluna2</t>
+  </si>
+  <si>
+    <t>Coluna3</t>
+  </si>
+  <si>
+    <t>Coluna4</t>
+  </si>
+  <si>
+    <t>0126-015288</t>
+  </si>
+  <si>
+    <t>PENDENTE FATURAMENTO</t>
+  </si>
+  <si>
+    <t>CLIENTE</t>
+  </si>
+  <si>
+    <t>Concluída no Field antes de entrar no hub</t>
+  </si>
+  <si>
+    <t>No Field a atividade já está concluída. O hub só traz do Field as OS do tipo "Atividade Spot" com atividade pendente, agendada ou em andamento (critério combinado em 15/09). Ela foi concluída sem ter entrado no hub, então ficou de fora.</t>
+  </si>
+  <si>
+    <t>Se vocês querem acompanhar no hub também as OS já concluídas no Field (por exemplo, até o faturamento), o critério precisa mudar. Fica para decidirmos juntos.</t>
+  </si>
+  <si>
+    <t>0226-009618</t>
+  </si>
+  <si>
+    <t>0326-009215</t>
+  </si>
+  <si>
+    <t>0326-009444</t>
+  </si>
+  <si>
+    <t>0326-010522</t>
+  </si>
+  <si>
+    <t>0326-012374</t>
+  </si>
+  <si>
+    <t>0326-012395</t>
+  </si>
+  <si>
+    <t>0326-018781</t>
+  </si>
+  <si>
+    <t>0426-012516</t>
+  </si>
+  <si>
+    <t>0426-016925</t>
+  </si>
+  <si>
+    <t>0426-016931</t>
+  </si>
+  <si>
+    <t>0426-017866</t>
+  </si>
+  <si>
+    <t>0526-008051</t>
+  </si>
+  <si>
+    <t>0526-013041</t>
+  </si>
+  <si>
+    <t>0526-013810</t>
+  </si>
+  <si>
+    <t>0526-016397</t>
+  </si>
+  <si>
+    <t>0526-016495</t>
+  </si>
+  <si>
+    <t>0526-017199</t>
+  </si>
+  <si>
+    <t>Tipo "Manutenção Corretiva" no Field</t>
+  </si>
+  <si>
+    <t>No Field esta OS é do tipo "Manutenção Corretiva" (atividade concluída). O hub só traz do Field as OS do tipo "Atividade Spot" com atividade pendente, agendada ou em andamento (critério combinado em 15/09).</t>
+  </si>
+  <si>
+    <t>Se é obra, trocar o tipo para "Atividade Spot". Como a atividade já está concluída, mesmo assim não entraria (ver as concluídas).</t>
+  </si>
+  <si>
+    <t>0526-018908</t>
+  </si>
+  <si>
+    <t>0526-019340</t>
+  </si>
+  <si>
+    <t>0526-019250</t>
+  </si>
+  <si>
+    <t>0626-004129</t>
+  </si>
+  <si>
+    <t>0626-004183</t>
+  </si>
+  <si>
+    <t>0626-004592</t>
+  </si>
+  <si>
+    <t>0626-005012</t>
+  </si>
+  <si>
+    <t>0626-005068</t>
+  </si>
+  <si>
+    <t>0626-005488</t>
+  </si>
+  <si>
+    <t>0626-005880</t>
+  </si>
+  <si>
+    <t>0626-006632</t>
+  </si>
+  <si>
+    <t>0726-009420</t>
+  </si>
+  <si>
+    <t>0726-010838</t>
+  </si>
+  <si>
+    <t>0726-011532</t>
+  </si>
+  <si>
+    <t>0726-012445</t>
+  </si>
+  <si>
+    <t>0726-013344</t>
+  </si>
+  <si>
+    <t>0726-015135</t>
+  </si>
+  <si>
+    <t>0726-018016</t>
+  </si>
+  <si>
+    <t>0726-018751</t>
+  </si>
+  <si>
+    <t>0726-009288</t>
+  </si>
+  <si>
+    <t>FECHAR OS</t>
+  </si>
+  <si>
+    <t>0826-006388</t>
+  </si>
+  <si>
+    <t>0726-019011</t>
+  </si>
+  <si>
+    <t>0826-005453</t>
+  </si>
+  <si>
+    <t>Atividade "reportada" no Field</t>
+  </si>
+  <si>
+    <t>Na última atividade da OS no Field a situação é "reportada". O hub só traz do Field as OS do tipo "Atividade Spot" com atividade pendente, agendada ou em andamento (critério combinado em 15/09).</t>
+  </si>
+  <si>
+    <t>Se a obra continua, ajustar a situação da atividade no Field.</t>
+  </si>
+  <si>
+    <t>0826-007642</t>
+  </si>
+  <si>
+    <t>0926-011139</t>
+  </si>
+  <si>
+    <t>EXECUTADO - APROVAR OS</t>
+  </si>
+  <si>
+    <t>0826-009182</t>
+  </si>
+  <si>
+    <t>0826-007943</t>
+  </si>
+  <si>
+    <t>0826-006948</t>
+  </si>
+  <si>
+    <t>0826-011936</t>
+  </si>
+  <si>
+    <t>0826-007936</t>
+  </si>
+  <si>
+    <t>0826-008257</t>
+  </si>
+  <si>
+    <t>EXECUTAR</t>
+  </si>
+  <si>
+    <t>No Field esta OS é do tipo "Manutenção Corretiva" (atividade pendente). O hub só traz do Field as OS do tipo "Atividade Spot" com atividade pendente, agendada ou em andamento (critério combinado em 15/09).</t>
+  </si>
+  <si>
+    <t>Se é obra, trocar o tipo da OS no Field para "Atividade Spot". Ela entra no hub em poucos minutos.</t>
+  </si>
+  <si>
+    <t>SEM OS</t>
+  </si>
+  <si>
+    <t>EXECUTAR - APROVAR OS</t>
+  </si>
+  <si>
+    <t>Sem número de OS</t>
+  </si>
+  <si>
+    <t>A linha não tem número de OS, então não há como achar no Field nem no hub.</t>
+  </si>
+  <si>
+    <t>Informar o número da OS (ou a loja e a descrição) para conferirmos.</t>
+  </si>
+  <si>
+    <t>0926-011149</t>
+  </si>
+  <si>
+    <t>1125-010536</t>
+  </si>
+  <si>
+    <t>1125-015968</t>
+  </si>
+  <si>
+    <t>1125-016234</t>
+  </si>
+  <si>
+    <t>1125-016236</t>
+  </si>
+  <si>
+    <t>0826-009507</t>
+  </si>
+  <si>
+    <t>0926-010483</t>
+  </si>
+  <si>
+    <t>0726-017852</t>
+  </si>
+  <si>
+    <t>0926-010003</t>
+  </si>
+  <si>
+    <t>Tipo "Emergencial" no Field</t>
+  </si>
+  <si>
+    <t>No Field esta OS é do tipo "Emergencial" (atividade pendente). O hub só traz do Field as OS do tipo "Atividade Spot" com atividade pendente, agendada ou em andamento (critério combinado em 15/09).</t>
+  </si>
+  <si>
+    <t>0926-009636</t>
+  </si>
+  <si>
+    <t>0826-004429</t>
+  </si>
+  <si>
+    <t>0726-009714</t>
+  </si>
+  <si>
+    <t>0926-015838</t>
+  </si>
+  <si>
+    <t>1026-006815</t>
+  </si>
+  <si>
+    <t>1026-005832</t>
+  </si>
+  <si>
+    <t>1026-005925</t>
+  </si>
+  <si>
+    <t>0526-019295</t>
+  </si>
+  <si>
+    <t>Não existe no Field</t>
+  </si>
+  <si>
+    <t>Não há OS com esse número no Field. Procuramos em todas as OS, inclusive arquivadas.</t>
+  </si>
+  <si>
+    <t>Conferir o número da OS no controle.</t>
+  </si>
+  <si>
+    <t>0626-003845</t>
+  </si>
+  <si>
+    <t>Não há OS com esse número no Field. Procuramos em todas as OS, inclusive arquivadas. Existe uma 0826-003845 no Field: pode ser erro de digitação no mês.</t>
+  </si>
+  <si>
+    <t>0726-017988</t>
+  </si>
+  <si>
+    <t>Está nos dois</t>
+  </si>
+  <si>
+    <t>Existe no Field (Atividade Spot, pendente) e entrou no hub hoje, 15/10, às 15h10, quando a atividade ficou pendente no Field. Na hora da conferência ainda não tinha entrado.</t>
+  </si>
+  <si>
+    <t>Nada a fazer. Já aparece no hub.</t>
+  </si>
+  <si>
+    <t>0726-018834</t>
+  </si>
+  <si>
+    <t>Tipo "Manutenção Corretiva" no Field, e a atividade está arquivada. Por isso não aparece no relatório do Field nem no hub.</t>
+  </si>
+  <si>
+    <t>Se a obra continua, desarquivar a atividade e conferir o tipo da OS no Field.</t>
+  </si>
+  <si>
+    <t>0726-018624</t>
+  </si>
+  <si>
+    <t>0726-017515</t>
+  </si>
+  <si>
+    <t>0726-018710</t>
+  </si>
+  <si>
+    <t>0726-017712</t>
+  </si>
+  <si>
+    <t>0726-018684</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -146,9 +474,6 @@
     <font>
       <b/>
       <color rgb="FFFFFFFF"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
   <fills count="3">
@@ -176,15 +501,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -531,8 +853,8 @@
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="16" customWidth="1"/>
-    <col min="5" max="5" width="24" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
     <col min="6" max="6" width="70" customWidth="1"/>
     <col min="7" max="7" width="55" customWidth="1"/>
   </cols>
@@ -570,7 +892,7 @@
       <c r="C2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="D2" s="2" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="2" t="s">
@@ -593,22 +915,22 @@
       <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
@@ -616,22 +938,22 @@
       <c r="C4" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>18</v>
+      <c r="D4" s="2" t="s">
+        <v>19</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>8</v>
@@ -639,22 +961,22 @@
       <c r="C5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>22</v>
+      <c r="D5" s="2" t="s">
+        <v>23</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>8</v>
@@ -662,22 +984,22 @@
       <c r="C6" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>26</v>
+      <c r="D6" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>8</v>
@@ -685,22 +1007,22 @@
       <c r="C7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>30</v>
+      <c r="D7" s="2" t="s">
+        <v>31</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
@@ -708,17 +1030,17 @@
       <c r="C8" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>34</v>
+      <c r="D8" s="2" t="s">
+        <v>35</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -730,23 +1052,1810 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="100" customWidth="1"/>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="70" customWidth="1"/>
+    <col min="7" max="7" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="B1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="41" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A42" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="43" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A43" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F43" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F45" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="B46" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E46" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F46" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="47" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="B47" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D47" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E47" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F47" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D48" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E48" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F48" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="B51" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="C51" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="52" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D52" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E52" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F52" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E53" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F53" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G53" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="54" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A54" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="C54" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D54" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E54" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F54" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A55" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="C55" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E55" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F55" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A56" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B56" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="C56" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D56" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E56" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F56" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A57" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="C57" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D57" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E57" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="B58" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C58" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E58" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F58" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A59" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="C59" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D59" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E59" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C60" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D60" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E60" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F60" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A61" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="B61" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C61" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D61" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E61" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B62" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C62" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D62" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E62" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A63" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B63" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C63" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D63" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E63" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B64" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C64" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D64" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E64" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F64" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="65" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A65" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B65" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="C65" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D65" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E65" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F65" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B66" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="C66" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D66" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E66" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F66" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="67" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B67" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C67" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D67" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E67" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F67" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>106</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="2" width="14" customWidth="1"/>
+    <col min="3" max="3" width="24" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="6" width="70" customWidth="1"/>
+    <col min="7" max="7" width="55" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>142</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>